<commit_message>
Added 9-24-2026 WNBA Results
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -27190,6 +27190,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H636" t="n">
+        <v>95</v>
+      </c>
+      <c r="I636" t="n">
+        <v>84</v>
+      </c>
+      <c r="J636" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="637">
       <c r="A637" s="1" t="n">
@@ -27223,6 +27232,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H637" t="n">
+        <v>84</v>
+      </c>
+      <c r="I637" t="n">
+        <v>95</v>
+      </c>
+      <c r="J637" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="638">
       <c r="A638" s="1" t="n">
@@ -27256,6 +27274,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H638" t="n">
+        <v>86</v>
+      </c>
+      <c r="I638" t="n">
+        <v>87</v>
+      </c>
+      <c r="J638" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="639">
       <c r="A639" s="1" t="n">
@@ -27289,6 +27316,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H639" t="n">
+        <v>87</v>
+      </c>
+      <c r="I639" t="n">
+        <v>86</v>
+      </c>
+      <c r="J639" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="640">
       <c r="A640" s="1" t="n">
@@ -27322,6 +27358,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H640" t="n">
+        <v>85</v>
+      </c>
+      <c r="I640" t="n">
+        <v>97</v>
+      </c>
+      <c r="J640" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="641">
       <c r="A641" s="1" t="n">
@@ -27355,6 +27400,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H641" t="n">
+        <v>97</v>
+      </c>
+      <c r="I641" t="n">
+        <v>85</v>
+      </c>
+      <c r="J641" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="642">
       <c r="A642" s="1" t="n">
@@ -27388,6 +27442,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H642" t="n">
+        <v>77</v>
+      </c>
+      <c r="I642" t="n">
+        <v>96</v>
+      </c>
+      <c r="J642" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="643">
       <c r="A643" s="1" t="n">
@@ -27421,6 +27484,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H643" t="n">
+        <v>96</v>
+      </c>
+      <c r="I643" t="n">
+        <v>77</v>
+      </c>
+      <c r="J643" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="644">
       <c r="A644" s="1" t="n">
@@ -27454,6 +27526,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H644" t="n">
+        <v>79</v>
+      </c>
+      <c r="I644" t="n">
+        <v>89</v>
+      </c>
+      <c r="J644" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="645">
       <c r="A645" s="1" t="n">
@@ -27487,6 +27568,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H645" t="n">
+        <v>89</v>
+      </c>
+      <c r="I645" t="n">
+        <v>79</v>
+      </c>
+      <c r="J645" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="646">
       <c r="A646" s="1" t="n">
@@ -27520,6 +27610,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H646" t="n">
+        <v>82</v>
+      </c>
+      <c r="I646" t="n">
+        <v>90</v>
+      </c>
+      <c r="J646" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="647">
       <c r="A647" s="1" t="n">
@@ -27553,6 +27652,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H647" t="n">
+        <v>90</v>
+      </c>
+      <c r="I647" t="n">
+        <v>82</v>
+      </c>
+      <c r="J647" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="648">
       <c r="A648" s="1" t="n">
@@ -27586,6 +27694,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H648" t="n">
+        <v>69</v>
+      </c>
+      <c r="I648" t="n">
+        <v>79</v>
+      </c>
+      <c r="J648" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="649">
       <c r="A649" s="1" t="n">
@@ -27619,6 +27736,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H649" t="n">
+        <v>79</v>
+      </c>
+      <c r="I649" t="n">
+        <v>69</v>
+      </c>
+      <c r="J649" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="650">
       <c r="A650" s="1" t="n">
@@ -27652,6 +27778,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H650" t="n">
+        <v>83</v>
+      </c>
+      <c r="I650" t="n">
+        <v>65</v>
+      </c>
+      <c r="J650" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="651">
       <c r="A651" s="1" t="n">
@@ -27685,6 +27820,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H651" t="n">
+        <v>65</v>
+      </c>
+      <c r="I651" t="n">
+        <v>83</v>
+      </c>
+      <c r="J651" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="652">
       <c r="A652" s="1" t="n">
@@ -27718,6 +27862,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H652" t="n">
+        <v>103</v>
+      </c>
+      <c r="I652" t="n">
+        <v>91</v>
+      </c>
+      <c r="J652" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="653">
       <c r="A653" s="1" t="n">
@@ -27751,6 +27904,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H653" t="n">
+        <v>91</v>
+      </c>
+      <c r="I653" t="n">
+        <v>103</v>
+      </c>
+      <c r="J653" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="654">
       <c r="A654" s="1" t="n">
@@ -27784,6 +27946,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H654" t="n">
+        <v>81</v>
+      </c>
+      <c r="I654" t="n">
+        <v>95</v>
+      </c>
+      <c r="J654" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="655">
       <c r="A655" s="1" t="n">
@@ -27817,6 +27988,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H655" t="n">
+        <v>95</v>
+      </c>
+      <c r="I655" t="n">
+        <v>81</v>
+      </c>
+      <c r="J655" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="656">
       <c r="A656" s="1" t="n">
@@ -27850,6 +28030,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H656" t="n">
+        <v>76</v>
+      </c>
+      <c r="I656" t="n">
+        <v>75</v>
+      </c>
+      <c r="J656" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="657">
       <c r="A657" s="1" t="n">
@@ -27883,6 +28072,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H657" t="n">
+        <v>75</v>
+      </c>
+      <c r="I657" t="n">
+        <v>76</v>
+      </c>
+      <c r="J657" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="658">
       <c r="A658" s="1" t="n">
@@ -27916,6 +28114,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H658" t="n">
+        <v>66</v>
+      </c>
+      <c r="I658" t="n">
+        <v>86</v>
+      </c>
+      <c r="J658" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="659">
       <c r="A659" s="1" t="n">
@@ -27949,6 +28156,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H659" t="n">
+        <v>86</v>
+      </c>
+      <c r="I659" t="n">
+        <v>66</v>
+      </c>
+      <c r="J659" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="660">
       <c r="A660" s="1" t="n">
@@ -27982,6 +28198,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H660" t="n">
+        <v>100</v>
+      </c>
+      <c r="I660" t="n">
+        <v>82</v>
+      </c>
+      <c r="J660" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="661">
       <c r="A661" s="1" t="n">
@@ -28015,6 +28240,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H661" t="n">
+        <v>82</v>
+      </c>
+      <c r="I661" t="n">
+        <v>100</v>
+      </c>
+      <c r="J661" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="662">
       <c r="A662" s="1" t="n">
@@ -28048,6 +28282,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H662" t="n">
+        <v>93</v>
+      </c>
+      <c r="I662" t="n">
+        <v>101</v>
+      </c>
+      <c r="J662" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="663">
       <c r="A663" s="1" t="n">
@@ -28080,6 +28323,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H663" t="n">
+        <v>101</v>
+      </c>
+      <c r="I663" t="n">
+        <v>93</v>
+      </c>
+      <c r="J663" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Incorrect Playoff Date
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\TRACERsports\DBs\wnba\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49AE1844-FD48-4B16-B3A8-1D32E66BFDDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47E239E1-8E7D-432D-BF2A-6C8E2FB06728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22084,7 +22084,7 @@
     </row>
     <row r="676" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A676" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B676">
         <v>2026</v>
@@ -22107,7 +22107,7 @@
     </row>
     <row r="677" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A677" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B677">
         <v>2026</v>
@@ -22130,7 +22130,7 @@
     </row>
     <row r="678" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A678" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B678">
         <v>2026</v>
@@ -22153,7 +22153,7 @@
     </row>
     <row r="679" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A679" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B679">
         <v>2026</v>

</xml_diff>

<commit_message>
Added WNBA Playoff Results for 9-30-2026 Pt 1
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -129,8 +129,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J681" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:J681"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J683" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:J683"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Date" dataDxfId="0"/>
     <tableColumn id="2" name="Season"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J681"/>
+  <dimension ref="A1:J683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.5"/>
   <cols>
     <col width="9.9140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -28844,6 +28844,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H676" t="n">
+        <v>93</v>
+      </c>
+      <c r="I676" t="n">
+        <v>75</v>
+      </c>
+      <c r="J676" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="677">
       <c r="A677" s="1" t="n">
@@ -28875,6 +28884,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H677" t="n">
+        <v>75</v>
+      </c>
+      <c r="I677" t="n">
+        <v>93</v>
+      </c>
+      <c r="J677" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="678">
       <c r="A678" s="1" t="n">
@@ -28995,6 +29013,68 @@
         </is>
       </c>
       <c r="G681" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="1" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B682" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D682" t="n">
+        <v>2</v>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>NYL</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="1" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B683" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D683" t="n">
+        <v>2</v>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>NYL</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>

<commit_message>
Fixed Broken WNBA Playoff Games
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -129,8 +129,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J683" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:J683"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J685" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:J685"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Date" dataDxfId="0"/>
     <tableColumn id="2" name="Season"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J683"/>
+  <dimension ref="A1:J685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.5"/>
   <cols>
     <col width="9.9140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -28924,6 +28924,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H678" t="n">
+        <v>100</v>
+      </c>
+      <c r="I678" t="n">
+        <v>108</v>
+      </c>
+      <c r="J678" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="679">
       <c r="A679" s="1" t="n">
@@ -28955,6 +28964,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H679" t="n">
+        <v>108</v>
+      </c>
+      <c r="I679" t="n">
+        <v>100</v>
+      </c>
+      <c r="J679" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="680">
       <c r="A680" s="1" t="n">
@@ -29075,6 +29093,68 @@
         </is>
       </c>
       <c r="G683" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B684" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D684" t="n">
+        <v>1</v>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>GSV</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B685" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D685" t="n">
+        <v>1</v>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>GSV</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>

<commit_message>
Added WNBA Playoff Games for 10-2-2026
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -29004,6 +29004,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H680" t="n">
+        <v>94</v>
+      </c>
+      <c r="I680" t="n">
+        <v>83</v>
+      </c>
+      <c r="J680" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="681">
       <c r="A681" s="1" t="n">
@@ -29034,6 +29043,15 @@
         <is>
           <t>A</t>
         </is>
+      </c>
+      <c r="H681" t="n">
+        <v>83</v>
+      </c>
+      <c r="I681" t="n">
+        <v>94</v>
+      </c>
+      <c r="J681" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="682">

</xml_diff>

<commit_message>
Added WNBA Playoff Results for 10-2-2026
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -129,8 +129,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J685" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:J685"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J687" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:J687"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Date" dataDxfId="0"/>
     <tableColumn id="2" name="Season"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J685"/>
+  <dimension ref="A1:J687"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.5"/>
   <cols>
     <col width="9.9140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -29146,6 +29146,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H684" t="n">
+        <v>77</v>
+      </c>
+      <c r="I684" t="n">
+        <v>73</v>
+      </c>
+      <c r="J684" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="685">
       <c r="A685" s="1" t="n">
@@ -29173,6 +29182,77 @@
         </is>
       </c>
       <c r="G685" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H685" t="n">
+        <v>73</v>
+      </c>
+      <c r="I685" t="n">
+        <v>77</v>
+      </c>
+      <c r="J685" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="1" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B686" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D686" t="n">
+        <v>2</v>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>GSV</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>LVA</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="1" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B687" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D687" t="n">
+        <v>2</v>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>LVA</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>GSV</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>

<commit_message>
Added 10-7-2026 WNBA Playoff Results
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -29327,6 +29327,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H688" t="n">
+        <v>101</v>
+      </c>
+      <c r="I688" t="n">
+        <v>98</v>
+      </c>
+      <c r="J688" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="689">
       <c r="A689" s="1" t="n">
@@ -29358,6 +29367,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H689" t="n">
+        <v>98</v>
+      </c>
+      <c r="I689" t="n">
+        <v>101</v>
+      </c>
+      <c r="J689" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="690">
       <c r="A690" s="1" t="n">
@@ -29389,6 +29407,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H690" t="n">
+        <v>83</v>
+      </c>
+      <c r="I690" t="n">
+        <v>81</v>
+      </c>
+      <c r="J690" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="691">
       <c r="A691" s="1" t="n">
@@ -29419,6 +29446,15 @@
         <is>
           <t>A</t>
         </is>
+      </c>
+      <c r="H691" t="n">
+        <v>81</v>
+      </c>
+      <c r="I691" t="n">
+        <v>83</v>
+      </c>
+      <c r="J691" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="692">

</xml_diff>

<commit_message>
Added WNBA Playoff Results for Oct 9, 2026
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -29487,6 +29487,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H692" t="n">
+        <v>85</v>
+      </c>
+      <c r="I692" t="n">
+        <v>83</v>
+      </c>
+      <c r="J692" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="693">
       <c r="A693" s="1" t="n">
@@ -29518,6 +29527,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H693" t="n">
+        <v>83</v>
+      </c>
+      <c r="I693" t="n">
+        <v>85</v>
+      </c>
+      <c r="J693" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="694">
       <c r="A694" s="1" t="n">
@@ -29549,6 +29567,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H694" t="n">
+        <v>87</v>
+      </c>
+      <c r="I694" t="n">
+        <v>77</v>
+      </c>
+      <c r="J694" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="695">
       <c r="A695" s="1" t="n">
@@ -29579,6 +29606,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H695" t="n">
+        <v>77</v>
+      </c>
+      <c r="I695" t="n">
+        <v>87</v>
+      </c>
+      <c r="J695" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added WNBA Playoff Results for Oct 19, 2026
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -29727,6 +29727,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H698" t="n">
+        <v>79</v>
+      </c>
+      <c r="I698" t="n">
+        <v>65</v>
+      </c>
+      <c r="J698" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="699">
       <c r="A699" s="1" t="n">
@@ -29757,6 +29766,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H699" t="n">
+        <v>65</v>
+      </c>
+      <c r="I699" t="n">
+        <v>79</v>
+      </c>
+      <c r="J699" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="700">

</xml_diff>

<commit_message>
Added WNBA Playoff Results for Oct 21, 2026
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -129,8 +129,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J703" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:J703"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J705" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:J705"/>
   <sortState ref="A2:J687">
     <sortCondition ref="A682:A687"/>
   </sortState>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J703"/>
+  <dimension ref="A1:J705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.5"/>
   <cols>
     <col width="9.9140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -29901,6 +29901,86 @@
         </is>
       </c>
     </row>
+    <row r="704">
+      <c r="A704" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B704" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D704" t="n">
+        <v>3</v>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>GSV</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="H704" t="n">
+        <v>97</v>
+      </c>
+      <c r="I704" t="n">
+        <v>71</v>
+      </c>
+      <c r="J704" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B705" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D705" t="n">
+        <v>3</v>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>GSV</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H705" t="n">
+        <v>71</v>
+      </c>
+      <c r="I705" t="n">
+        <v>97</v>
+      </c>
+      <c r="J705" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>